<commit_message>
Corrections to enable bootstrapping
</commit_message>
<xml_diff>
--- a/input/projections_fertility.xlsx
+++ b/input/projections_fertility.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryk\git\labsim\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E268E892-D14D-4480-8A90-D0AA4EA574E7}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D2AC8B9-4751-8F42-B10D-F30EA2EB9805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3405" yWindow="1320" windowWidth="31350" windowHeight="16950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1320" windowWidth="30240" windowHeight="16960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
-    <sheet name="UK_FertilityByYear" sheetId="3" r:id="rId2"/>
-    <sheet name="IT_FertilityByYear" sheetId="4" r:id="rId3"/>
+    <sheet name="FertilityByYear" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -66,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="88">
   <si>
     <t/>
   </si>
@@ -402,9 +401,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -442,7 +441,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -548,7 +547,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -690,7 +689,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -699,9 +698,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E78"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -709,7 +708,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -717,7 +716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
         <v>87</v>
       </c>
@@ -725,7 +724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -733,7 +732,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -741,7 +740,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -749,7 +748,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -766,7 +765,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A8" t="s">
         <v>10</v>
       </c>
@@ -784,7 +783,7 @@
         <v>67.666666666666671</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -802,7 +801,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -820,7 +819,7 @@
         <v>60.333333333333336</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A11" t="s">
         <v>16</v>
       </c>
@@ -838,7 +837,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -856,7 +855,7 @@
         <v>56.333333333333336</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A13" t="s">
         <v>18</v>
       </c>
@@ -874,7 +873,7 @@
         <v>58.666666666666664</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A14" t="s">
         <v>19</v>
       </c>
@@ -892,7 +891,7 @@
         <v>62.333333333333336</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -910,7 +909,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A16" t="s">
         <v>21</v>
       </c>
@@ -928,7 +927,7 @@
         <v>61.000000000000007</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A17" t="s">
         <v>22</v>
       </c>
@@ -946,7 +945,7 @@
         <v>59.333333333333336</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A18" t="s">
         <v>23</v>
       </c>
@@ -964,7 +963,7 @@
         <v>59.000000000000007</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A19" t="s">
         <v>24</v>
       </c>
@@ -982,7 +981,7 @@
         <v>59.000000000000007</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A20" t="s">
         <v>25</v>
       </c>
@@ -1000,7 +999,7 @@
         <v>59.666666666666664</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A21" t="s">
         <v>26</v>
       </c>
@@ -1018,7 +1017,7 @@
         <v>59.333333333333336</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A22" t="s">
         <v>27</v>
       </c>
@@ -1036,7 +1035,7 @@
         <v>60.333333333333336</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A23" t="s">
         <v>28</v>
       </c>
@@ -1054,7 +1053,7 @@
         <v>60.666666666666664</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A24" t="s">
         <v>29</v>
       </c>
@@ -1072,7 +1071,7 @@
         <v>59.666666666666664</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A25" t="s">
         <v>30</v>
       </c>
@@ -1090,7 +1089,7 @@
         <v>61.000000000000007</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A26" t="s">
         <v>31</v>
       </c>
@@ -1108,7 +1107,7 @@
         <v>60.666666666666664</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A27" t="s">
         <v>32</v>
       </c>
@@ -1126,7 +1125,7 @@
         <v>59.666666666666664</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A28" t="s">
         <v>33</v>
       </c>
@@ -1144,7 +1143,7 @@
         <v>58.666666666666664</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A29" t="s">
         <v>34</v>
       </c>
@@ -1162,7 +1161,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A30" t="s">
         <v>35</v>
       </c>
@@ -1180,7 +1179,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A31" t="s">
         <v>36</v>
       </c>
@@ -1198,7 +1197,7 @@
         <v>57.666666666666664</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A32" t="s">
         <v>37</v>
       </c>
@@ -1216,7 +1215,7 @@
         <v>57.333333333333336</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A33" t="s">
         <v>38</v>
       </c>
@@ -1234,7 +1233,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A34" t="s">
         <v>39</v>
       </c>
@@ -1252,7 +1251,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A35" t="s">
         <v>40</v>
       </c>
@@ -1270,7 +1269,7 @@
         <v>54.666666666666664</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A36" t="s">
         <v>41</v>
       </c>
@@ -1288,7 +1287,7 @@
         <v>54.333333333333329</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A37" t="s">
         <v>42</v>
       </c>
@@ -1306,7 +1305,7 @@
         <v>54.333333333333329</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A38" t="s">
         <v>43</v>
       </c>
@@ -1324,7 +1323,7 @@
         <v>56.666666666666664</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A39" t="s">
         <v>44</v>
       </c>
@@ -1342,7 +1341,7 @@
         <v>58.666666666666664</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A40" t="s">
         <v>45</v>
       </c>
@@ -1360,7 +1359,7 @@
         <v>58.666666666666664</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A41" t="s">
         <v>46</v>
       </c>
@@ -1378,7 +1377,7 @@
         <v>60.666666666666664</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A42" t="s">
         <v>47</v>
       </c>
@@ -1396,7 +1395,7 @@
         <v>62.333333333333336</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A43" t="s">
         <v>48</v>
       </c>
@@ -1414,7 +1413,7 @@
         <v>63.666666666666664</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A44" t="s">
         <v>49</v>
       </c>
@@ -1432,7 +1431,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A45" t="s">
         <v>50</v>
       </c>
@@ -1450,7 +1449,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A46" t="s">
         <v>51</v>
       </c>
@@ -1468,7 +1467,7 @@
         <v>63.666666666666664</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A47" t="s">
         <v>52</v>
       </c>
@@ -1486,7 +1485,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A48" t="s">
         <v>53</v>
       </c>
@@ -1504,7 +1503,7 @@
         <v>61.000000000000007</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A49" t="s">
         <v>54</v>
       </c>
@@ -1522,7 +1521,7 @@
         <v>60.666666666666664</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A50" t="s">
         <v>55</v>
       </c>
@@ -1540,7 +1539,7 @@
         <v>60.000000000000007</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A51" t="s">
         <v>56</v>
       </c>
@@ -1558,7 +1557,7 @@
         <v>59.666666666666664</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A52" t="s">
         <v>57</v>
       </c>
@@ -1576,7 +1575,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A53" t="s">
         <v>58</v>
       </c>
@@ -1594,7 +1593,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A54" t="s">
         <v>59</v>
       </c>
@@ -1612,7 +1611,7 @@
         <v>55.333333333333329</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A55" t="s">
         <v>60</v>
       </c>
@@ -1630,7 +1629,7 @@
         <v>55.333333333333329</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A56" t="s">
         <v>61</v>
       </c>
@@ -1648,7 +1647,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A57" t="s">
         <v>62</v>
       </c>
@@ -1666,7 +1665,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A58" t="s">
         <v>63</v>
       </c>
@@ -1684,7 +1683,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A59" t="s">
         <v>64</v>
       </c>
@@ -1702,7 +1701,7 @@
         <v>55.333333333333329</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A60" t="s">
         <v>65</v>
       </c>
@@ -1720,7 +1719,7 @@
         <v>55.666666666666664</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A61" t="s">
         <v>66</v>
       </c>
@@ -1738,7 +1737,7 @@
         <v>55.666666666666664</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A62" t="s">
         <v>67</v>
       </c>
@@ -1756,7 +1755,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A63" t="s">
         <v>68</v>
       </c>
@@ -1774,7 +1773,7 @@
         <v>56.333333333333336</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A64" t="s">
         <v>69</v>
       </c>
@@ -1792,7 +1791,7 @@
         <v>56.666666666666664</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A65" t="s">
         <v>70</v>
       </c>
@@ -1810,7 +1809,7 @@
         <v>56.666666666666664</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A66" t="s">
         <v>71</v>
       </c>
@@ -1828,7 +1827,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A67" t="s">
         <v>72</v>
       </c>
@@ -1846,7 +1845,7 @@
         <v>57.333333333333336</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A68" t="s">
         <v>73</v>
       </c>
@@ -1864,7 +1863,7 @@
         <v>57.666666666666664</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A69" t="s">
         <v>74</v>
       </c>
@@ -1882,7 +1881,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A70" t="s">
         <v>75</v>
       </c>
@@ -1900,7 +1899,7 @@
         <v>58.333333333333336</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A71" t="s">
         <v>76</v>
       </c>
@@ -1918,7 +1917,7 @@
         <v>58.333333333333336</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A72" t="s">
         <v>77</v>
       </c>
@@ -1936,7 +1935,7 @@
         <v>58.666666666666664</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A73" t="s">
         <v>78</v>
       </c>
@@ -1954,7 +1953,7 @@
         <v>59.000000000000007</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A74" t="s">
         <v>79</v>
       </c>
@@ -1972,7 +1971,7 @@
         <v>59.000000000000007</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A75" t="s">
         <v>80</v>
       </c>
@@ -1990,7 +1989,7 @@
         <v>59.333333333333336</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A76" t="s">
         <v>81</v>
       </c>
@@ -2008,7 +2007,7 @@
         <v>59.333333333333336</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A77" t="s">
         <v>82</v>
       </c>
@@ -2026,7 +2025,7 @@
         <v>59.333333333333336</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A78" t="s">
         <v>83</v>
       </c>
@@ -2055,9 +2054,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CC6C525-5E56-43D0-8485-7B36B4DC93F6}">
   <dimension ref="A1:BT2"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1" spans="1:72" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:72" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
         <v>85</v>
       </c>
@@ -2275,453 +2274,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="2" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>84</v>
-      </c>
-      <c r="B2">
-        <v>67.666666666666671</v>
-      </c>
-      <c r="C2">
-        <v>64</v>
-      </c>
-      <c r="D2">
-        <v>60.333333333333336</v>
-      </c>
-      <c r="E2">
-        <v>58</v>
-      </c>
-      <c r="F2">
-        <v>56.333333333333336</v>
-      </c>
-      <c r="G2">
-        <v>58.666666666666664</v>
-      </c>
-      <c r="H2">
-        <v>62.333333333333336</v>
-      </c>
-      <c r="I2">
-        <v>63</v>
-      </c>
-      <c r="J2">
-        <v>61.000000000000007</v>
-      </c>
-      <c r="K2">
-        <v>59.333333333333336</v>
-      </c>
-      <c r="L2">
-        <v>59.000000000000007</v>
-      </c>
-      <c r="M2">
-        <v>59.000000000000007</v>
-      </c>
-      <c r="N2">
-        <v>59.666666666666664</v>
-      </c>
-      <c r="O2">
-        <v>59.333333333333336</v>
-      </c>
-      <c r="P2">
-        <v>60.333333333333336</v>
-      </c>
-      <c r="Q2">
-        <v>60.666666666666664</v>
-      </c>
-      <c r="R2">
-        <v>59.666666666666664</v>
-      </c>
-      <c r="S2">
-        <v>61.000000000000007</v>
-      </c>
-      <c r="T2">
-        <v>60.666666666666664</v>
-      </c>
-      <c r="U2">
-        <v>59.666666666666664</v>
-      </c>
-      <c r="V2">
-        <v>58.666666666666664</v>
-      </c>
-      <c r="W2">
-        <v>58</v>
-      </c>
-      <c r="X2">
-        <v>57</v>
-      </c>
-      <c r="Y2">
-        <v>57.666666666666664</v>
-      </c>
-      <c r="Z2">
-        <v>57.333333333333336</v>
-      </c>
-      <c r="AA2">
-        <v>57</v>
-      </c>
-      <c r="AB2">
-        <v>56</v>
-      </c>
-      <c r="AC2">
-        <v>54.666666666666664</v>
-      </c>
-      <c r="AD2">
-        <v>54.333333333333329</v>
-      </c>
-      <c r="AE2">
-        <v>54.333333333333329</v>
-      </c>
-      <c r="AF2">
-        <v>56.666666666666664</v>
-      </c>
-      <c r="AG2">
-        <v>58.666666666666664</v>
-      </c>
-      <c r="AH2">
-        <v>58.666666666666664</v>
-      </c>
-      <c r="AI2">
-        <v>60.666666666666664</v>
-      </c>
-      <c r="AJ2">
-        <v>62.333333333333336</v>
-      </c>
-      <c r="AK2">
-        <v>63.666666666666664</v>
-      </c>
-      <c r="AL2">
-        <v>63</v>
-      </c>
-      <c r="AM2">
-        <v>64</v>
-      </c>
-      <c r="AN2">
-        <v>63.666666666666664</v>
-      </c>
-      <c r="AO2">
-        <v>64</v>
-      </c>
-      <c r="AP2">
-        <v>61.000000000000007</v>
-      </c>
-      <c r="AQ2">
-        <v>60.666666666666664</v>
-      </c>
-      <c r="AR2">
-        <v>60.000000000000007</v>
-      </c>
-      <c r="AS2">
-        <v>59.666666666666664</v>
-      </c>
-      <c r="AT2">
-        <v>58</v>
-      </c>
-      <c r="AU2">
-        <v>56</v>
-      </c>
-      <c r="AV2">
-        <v>55.333333333333329</v>
-      </c>
-      <c r="AW2">
-        <v>55.333333333333329</v>
-      </c>
-      <c r="AX2">
-        <v>55</v>
-      </c>
-      <c r="AY2">
-        <v>55</v>
-      </c>
-      <c r="AZ2">
-        <v>55</v>
-      </c>
-      <c r="BA2">
-        <v>55.333333333333329</v>
-      </c>
-      <c r="BB2">
-        <v>55.666666666666664</v>
-      </c>
-      <c r="BC2">
-        <v>55.666666666666664</v>
-      </c>
-      <c r="BD2">
-        <v>56</v>
-      </c>
-      <c r="BE2">
-        <v>56.333333333333336</v>
-      </c>
-      <c r="BF2">
-        <v>56.666666666666664</v>
-      </c>
-      <c r="BG2">
-        <v>56.666666666666664</v>
-      </c>
-      <c r="BH2">
-        <v>57</v>
-      </c>
-      <c r="BI2">
-        <v>57.333333333333336</v>
-      </c>
-      <c r="BJ2">
-        <v>57.666666666666664</v>
-      </c>
-      <c r="BK2">
-        <v>58</v>
-      </c>
-      <c r="BL2">
-        <v>58.333333333333336</v>
-      </c>
-      <c r="BM2">
-        <v>58.333333333333336</v>
-      </c>
-      <c r="BN2">
-        <v>58.666666666666664</v>
-      </c>
-      <c r="BO2">
-        <v>59.000000000000007</v>
-      </c>
-      <c r="BP2">
-        <v>59.000000000000007</v>
-      </c>
-      <c r="BQ2">
-        <v>59.333333333333336</v>
-      </c>
-      <c r="BR2">
-        <v>59.333333333333336</v>
-      </c>
-      <c r="BS2">
-        <v>59.333333333333336</v>
-      </c>
-      <c r="BT2">
-        <v>59.333333333333336</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{331DBE6D-1954-4346-8599-CE9CA47D5F47}">
-  <dimension ref="A1:BT2"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
-  <sheetData>
-    <row r="1" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
-        <v>85</v>
-      </c>
-      <c r="B1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H1" t="s">
-        <v>19</v>
-      </c>
-      <c r="I1" t="s">
-        <v>20</v>
-      </c>
-      <c r="J1" t="s">
-        <v>21</v>
-      </c>
-      <c r="K1" t="s">
-        <v>22</v>
-      </c>
-      <c r="L1" t="s">
-        <v>23</v>
-      </c>
-      <c r="M1" t="s">
-        <v>24</v>
-      </c>
-      <c r="N1" t="s">
-        <v>25</v>
-      </c>
-      <c r="O1" t="s">
-        <v>26</v>
-      </c>
-      <c r="P1" t="s">
-        <v>27</v>
-      </c>
-      <c r="Q1" t="s">
-        <v>28</v>
-      </c>
-      <c r="R1" t="s">
-        <v>29</v>
-      </c>
-      <c r="S1" t="s">
-        <v>30</v>
-      </c>
-      <c r="T1" t="s">
-        <v>31</v>
-      </c>
-      <c r="U1" t="s">
-        <v>32</v>
-      </c>
-      <c r="V1" t="s">
-        <v>33</v>
-      </c>
-      <c r="W1" t="s">
-        <v>34</v>
-      </c>
-      <c r="X1" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y1" t="s">
-        <v>36</v>
-      </c>
-      <c r="Z1" t="s">
-        <v>37</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>38</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AG1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AI1" t="s">
-        <v>46</v>
-      </c>
-      <c r="AJ1" t="s">
-        <v>47</v>
-      </c>
-      <c r="AK1" t="s">
-        <v>48</v>
-      </c>
-      <c r="AL1" t="s">
-        <v>49</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AO1" t="s">
-        <v>52</v>
-      </c>
-      <c r="AP1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AQ1" t="s">
-        <v>54</v>
-      </c>
-      <c r="AR1" t="s">
-        <v>55</v>
-      </c>
-      <c r="AS1" t="s">
-        <v>56</v>
-      </c>
-      <c r="AT1" t="s">
-        <v>57</v>
-      </c>
-      <c r="AU1" t="s">
-        <v>58</v>
-      </c>
-      <c r="AV1" t="s">
-        <v>59</v>
-      </c>
-      <c r="AW1" t="s">
-        <v>60</v>
-      </c>
-      <c r="AX1" t="s">
-        <v>61</v>
-      </c>
-      <c r="AY1" t="s">
-        <v>62</v>
-      </c>
-      <c r="AZ1" t="s">
-        <v>63</v>
-      </c>
-      <c r="BA1" t="s">
-        <v>64</v>
-      </c>
-      <c r="BB1" t="s">
-        <v>65</v>
-      </c>
-      <c r="BC1" t="s">
-        <v>66</v>
-      </c>
-      <c r="BD1" t="s">
-        <v>67</v>
-      </c>
-      <c r="BE1" t="s">
-        <v>68</v>
-      </c>
-      <c r="BF1" t="s">
-        <v>69</v>
-      </c>
-      <c r="BG1" t="s">
-        <v>70</v>
-      </c>
-      <c r="BH1" t="s">
-        <v>71</v>
-      </c>
-      <c r="BI1" t="s">
-        <v>72</v>
-      </c>
-      <c r="BJ1" t="s">
-        <v>73</v>
-      </c>
-      <c r="BK1" t="s">
-        <v>74</v>
-      </c>
-      <c r="BL1" t="s">
-        <v>75</v>
-      </c>
-      <c r="BM1" t="s">
-        <v>76</v>
-      </c>
-      <c r="BN1" t="s">
-        <v>77</v>
-      </c>
-      <c r="BO1" t="s">
-        <v>78</v>
-      </c>
-      <c r="BP1" t="s">
-        <v>79</v>
-      </c>
-      <c r="BQ1" t="s">
-        <v>80</v>
-      </c>
-      <c r="BR1" t="s">
-        <v>81</v>
-      </c>
-      <c r="BS1" t="s">
-        <v>82</v>
-      </c>
-      <c r="BT1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="2" spans="1:72" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:72" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
         <v>84</v>
       </c>

</xml_diff>